<commit_message>
save 10 04 2026
</commit_message>
<xml_diff>
--- a/4 четверть_12_JavaScript_nodejs_Валидация данных.xlsx
+++ b/4 четверть_12_JavaScript_nodejs_Валидация данных.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE49BFC-1C55-4F4A-BF58-FA0E66D4F20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A8FB1F-8836-489C-965F-C320C3003C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-13875" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fastest validation" sheetId="14" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="385">
   <si>
     <t>Урок 1 часть 1</t>
   </si>
@@ -9290,17 +9290,406 @@
 }</t>
     </r>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>this.validatorSheme.validate(Object.assign({}, this.editedUserData)).map(i =&gt; {return i.path;});
+import Schema  from 'validate';</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>export const validatorSheme = new Schema</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">({
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UserMail</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: {
+       </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> required: true,
+        match: /^(([^&lt;&gt;()\[\]\\.,;:\s@"]+(\.[^&lt;&gt;()\[\]\\.,;:\s@"]+)*)|(".+"))@((\[[0-9]{1,3}\.[0-9]{1,3}\.[0-9]{1,3}\.[0-9]{1,3}\])|(([a-zA-Z\-0-9]+\.)+[a-zA-Z]{2,}))$///^([A-z0-9_\.-]+)@([A-z0-9_\.-]+)\.([A-z\.]{2,6})$/
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    },
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UserFirstName:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> {
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        required: true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    },
+   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> UserFamily:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> {
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        required: true,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    },
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>CloseDate:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> {
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        required: true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    },
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>UserPass:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> {
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        required: true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    },
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>newPass:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> {
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        required: false,
+        length: { min: 6, max: 32 },
+        match: /^(?=.*[a-z])(?=.*[A-Z])(?=.*[0-9]).{6,50}\b/
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    },
+   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> MailDistrib</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: {
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">        required: false,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+    }
+</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -9559,9 +9948,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -9572,57 +9961,57 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="6" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="3" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -9631,7 +10020,7 @@
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -9640,19 +10029,22 @@
     <xf numFmtId="49" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -9660,8 +10052,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{7B23FFB3-A72F-409B-B670-C03B7A66220A}"/>
+    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -10005,7 +10397,7 @@
       <c r="R3" s="1"/>
       <c r="U3" s="1"/>
     </row>
-    <row r="4" spans="1:22" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:22" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>375</v>
@@ -10013,7 +10405,9 @@
       <c r="C4" s="33" t="s">
         <v>377</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="34" t="s">
+        <v>384</v>
+      </c>
       <c r="G4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
@@ -12554,7 +12948,7 @@
       <c r="V3" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="10" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>